<commit_message>
review the test problems first thing on monday
</commit_message>
<xml_diff>
--- a/ProductFaangCodingPractice/ProblemSolvingList_ONLY_FOCUS.xlsx
+++ b/ProductFaangCodingPractice/ProblemSolvingList_ONLY_FOCUS.xlsx
@@ -29,7 +29,7 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
@@ -1319,6 +1319,12 @@
       <sz val="11"/>
       <color rgb="FFffffff"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -1359,12 +1365,6 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Open Sans"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
@@ -1484,7 +1484,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="34">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1495,22 +1495,22 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
@@ -1519,35 +1519,32 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="8" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="9" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1576,20 +1573,17 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="13" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1896,31 +1890,31 @@
   <dimension ref="A1:Y1002"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="32" width="15.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="32" width="12.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="33" width="5.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="32" width="36.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="34" width="20.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="34" width="19.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="35" width="39.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="34" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="32" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="31" width="15.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="31" width="12.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="32" width="5.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="31" width="36.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="33" width="20.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="33" width="19.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="31" width="39.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="33" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="31" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
@@ -3227,16 +3221,16 @@
       <c r="C35" s="2">
         <v>1</v>
       </c>
-      <c r="D35" s="21" t="s">
+      <c r="D35" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="E35" s="22" t="s">
+      <c r="E35" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F35" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="G35" s="23" t="s">
+      <c r="G35" s="22" t="s">
         <v>15</v>
       </c>
       <c r="H35" s="16" t="s">
@@ -3268,10 +3262,10 @@
       <c r="C36" s="2">
         <v>2</v>
       </c>
-      <c r="D36" s="21" t="s">
+      <c r="D36" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E36" s="22" t="s">
+      <c r="E36" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F36" s="17" t="s">
@@ -3307,10 +3301,10 @@
       <c r="C37" s="2">
         <v>3</v>
       </c>
-      <c r="D37" s="21" t="s">
+      <c r="D37" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E37" s="22" t="s">
+      <c r="E37" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F37" s="17" t="s">
@@ -3346,10 +3340,10 @@
       <c r="C38" s="2">
         <v>4</v>
       </c>
-      <c r="D38" s="21" t="s">
+      <c r="D38" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E38" s="22" t="s">
+      <c r="E38" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F38" s="17" t="s">
@@ -3387,10 +3381,10 @@
       <c r="C39" s="2">
         <v>5</v>
       </c>
-      <c r="D39" s="21" t="s">
+      <c r="D39" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E39" s="22" t="s">
+      <c r="E39" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F39" s="17" t="s">
@@ -3426,10 +3420,10 @@
       <c r="C40" s="2">
         <v>6</v>
       </c>
-      <c r="D40" s="21" t="s">
+      <c r="D40" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E40" s="22" t="s">
+      <c r="E40" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F40" s="17" t="s">
@@ -3470,7 +3464,7 @@
       <c r="D41" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="E41" s="22" t="s">
+      <c r="E41" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F41" s="19" t="s">
@@ -3565,7 +3559,7 @@
       <c r="D44" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="E44" s="22" t="s">
+      <c r="E44" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F44" s="15" t="s">
@@ -3606,7 +3600,7 @@
       <c r="D45" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E45" s="22" t="s">
+      <c r="E45" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F45" s="15" t="s">
@@ -3645,7 +3639,7 @@
       <c r="D46" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E46" s="22" t="s">
+      <c r="E46" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F46" s="15" t="s">
@@ -3684,7 +3678,7 @@
       <c r="D47" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E47" s="22" t="s">
+      <c r="E47" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F47" s="17" t="s">
@@ -3723,7 +3717,7 @@
       <c r="D48" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E48" s="22" t="s">
+      <c r="E48" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F48" s="17" t="s">
@@ -3762,7 +3756,7 @@
       <c r="D49" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E49" s="22" t="s">
+      <c r="E49" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F49" s="17" t="s">
@@ -3803,7 +3797,7 @@
       <c r="D50" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E50" s="22" t="s">
+      <c r="E50" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F50" s="17" t="s">
@@ -3842,7 +3836,7 @@
       <c r="D51" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E51" s="22" t="s">
+      <c r="E51" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F51" s="17" t="s">
@@ -3881,7 +3875,7 @@
       <c r="D52" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E52" s="22" t="s">
+      <c r="E52" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F52" s="19" t="s">
@@ -3920,7 +3914,7 @@
       <c r="D53" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E53" s="22" t="s">
+      <c r="E53" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F53" s="19" t="s">
@@ -3984,7 +3978,7 @@
       <c r="Y54" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="17.25">
-      <c r="A55" s="24"/>
+      <c r="A55" s="23"/>
       <c r="B55" s="6"/>
       <c r="C55" s="2"/>
       <c r="D55" s="5"/>
@@ -4038,7 +4032,7 @@
       <c r="Y56" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="17.25">
-      <c r="A57" s="25" t="s">
+      <c r="A57" s="24" t="s">
         <v>99</v>
       </c>
       <c r="B57" s="6" t="s">
@@ -4050,7 +4044,7 @@
       <c r="D57" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="E57" s="22" t="s">
+      <c r="E57" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F57" s="17" t="s">
@@ -4059,7 +4053,7 @@
       <c r="G57" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H57" s="26" t="s">
+      <c r="H57" s="25" t="s">
         <v>101</v>
       </c>
       <c r="I57" s="6"/>
@@ -4091,14 +4085,14 @@
       <c r="D58" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="E58" s="22" t="s">
+      <c r="E58" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F58" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G58" s="6"/>
-      <c r="H58" s="26" t="s">
+      <c r="H58" s="25" t="s">
         <v>103</v>
       </c>
       <c r="I58" s="6"/>
@@ -4130,7 +4124,7 @@
       <c r="D59" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="E59" s="22" t="s">
+      <c r="E59" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F59" s="17" t="s">
@@ -4139,7 +4133,7 @@
       <c r="G59" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H59" s="26" t="s">
+      <c r="H59" s="25" t="s">
         <v>105</v>
       </c>
       <c r="I59" s="6"/>
@@ -4171,14 +4165,14 @@
       <c r="D60" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="E60" s="22" t="s">
+      <c r="E60" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F60" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G60" s="6"/>
-      <c r="H60" s="26" t="s">
+      <c r="H60" s="25" t="s">
         <v>107</v>
       </c>
       <c r="I60" s="6"/>
@@ -4210,14 +4204,14 @@
       <c r="D61" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E61" s="22" t="s">
+      <c r="E61" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F61" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G61" s="6"/>
-      <c r="H61" s="26" t="s">
+      <c r="H61" s="25" t="s">
         <v>109</v>
       </c>
       <c r="I61" s="6"/>
@@ -4249,7 +4243,7 @@
       <c r="D62" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="E62" s="22" t="s">
+      <c r="E62" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F62" s="17" t="s">
@@ -4258,7 +4252,7 @@
       <c r="G62" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H62" s="26" t="s">
+      <c r="H62" s="25" t="s">
         <v>18</v>
       </c>
       <c r="I62" s="6"/>
@@ -4290,7 +4284,7 @@
       <c r="D63" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="E63" s="22" t="s">
+      <c r="E63" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F63" s="17" t="s">
@@ -4299,7 +4293,7 @@
       <c r="G63" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H63" s="27" t="s">
+      <c r="H63" s="26" t="s">
         <v>112</v>
       </c>
       <c r="I63" s="6"/>
@@ -4331,14 +4325,14 @@
       <c r="D64" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E64" s="22" t="s">
+      <c r="E64" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F64" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G64" s="6"/>
-      <c r="H64" s="26" t="s">
+      <c r="H64" s="25" t="s">
         <v>113</v>
       </c>
       <c r="I64" s="6"/>
@@ -4370,7 +4364,7 @@
       <c r="D65" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E65" s="22" t="s">
+      <c r="E65" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F65" s="19" t="s">
@@ -4379,7 +4373,7 @@
       <c r="G65" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H65" s="26" t="s">
+      <c r="H65" s="25" t="s">
         <v>115</v>
       </c>
       <c r="I65" s="6"/>
@@ -4411,7 +4405,7 @@
       <c r="D66" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="E66" s="22" t="s">
+      <c r="E66" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F66" s="19" t="s">
@@ -4420,7 +4414,7 @@
       <c r="G66" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H66" s="27" t="s">
+      <c r="H66" s="26" t="s">
         <v>117</v>
       </c>
       <c r="I66" s="6"/>
@@ -4452,14 +4446,14 @@
       <c r="D67" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E67" s="22" t="s">
+      <c r="E67" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F67" s="19" t="s">
         <v>63</v>
       </c>
       <c r="G67" s="6"/>
-      <c r="H67" s="27" t="s">
+      <c r="H67" s="26" t="s">
         <v>118</v>
       </c>
       <c r="I67" s="6"/>
@@ -4480,7 +4474,7 @@
       <c r="X67" s="1"/>
       <c r="Y67" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="19.5">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="2"/>
@@ -4507,7 +4501,7 @@
       <c r="X68" s="1"/>
       <c r="Y68" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="19.5">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="2"/>
@@ -4534,8 +4528,8 @@
       <c r="X69" s="1"/>
       <c r="Y69" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="17.25">
-      <c r="A70" s="25" t="s">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="19.5">
+      <c r="A70" s="24" t="s">
         <v>119</v>
       </c>
       <c r="B70" s="6" t="s">
@@ -4547,7 +4541,7 @@
       <c r="D70" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="E70" s="22" t="s">
+      <c r="E70" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F70" s="15" t="s">
@@ -4556,7 +4550,7 @@
       <c r="G70" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H70" s="26" t="s">
+      <c r="H70" s="25" t="s">
         <v>121</v>
       </c>
       <c r="I70" s="6"/>
@@ -4577,7 +4571,7 @@
       <c r="X70" s="1"/>
       <c r="Y70" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="19.5">
       <c r="A71" s="5"/>
       <c r="B71" s="6" t="s">
         <v>11</v>
@@ -4588,7 +4582,7 @@
       <c r="D71" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="E71" s="22" t="s">
+      <c r="E71" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F71" s="15" t="s">
@@ -4597,7 +4591,7 @@
       <c r="G71" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H71" s="26" t="s">
+      <c r="H71" s="25" t="s">
         <v>123</v>
       </c>
       <c r="I71" s="6"/>
@@ -4618,7 +4612,7 @@
       <c r="X71" s="1"/>
       <c r="Y71" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="19.5">
       <c r="A72" s="5"/>
       <c r="B72" s="6" t="s">
         <v>11</v>
@@ -4629,7 +4623,7 @@
       <c r="D72" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="E72" s="22" t="s">
+      <c r="E72" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F72" s="15" t="s">
@@ -4638,7 +4632,7 @@
       <c r="G72" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H72" s="26" t="s">
+      <c r="H72" s="25" t="s">
         <v>125</v>
       </c>
       <c r="I72" s="6"/>
@@ -4659,7 +4653,7 @@
       <c r="X72" s="1"/>
       <c r="Y72" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="19.5">
       <c r="A73" s="5"/>
       <c r="B73" s="6" t="s">
         <v>11</v>
@@ -4670,14 +4664,14 @@
       <c r="D73" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="E73" s="22" t="s">
+      <c r="E73" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F73" s="15" t="s">
         <v>14</v>
       </c>
       <c r="G73" s="6"/>
-      <c r="H73" s="26" t="s">
+      <c r="H73" s="25" t="s">
         <v>127</v>
       </c>
       <c r="I73" s="6"/>
@@ -4698,7 +4692,7 @@
       <c r="X73" s="1"/>
       <c r="Y73" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="19.5">
       <c r="A74" s="5"/>
       <c r="B74" s="6" t="s">
         <v>11</v>
@@ -4709,7 +4703,7 @@
       <c r="D74" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E74" s="22" t="s">
+      <c r="E74" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F74" s="15" t="s">
@@ -4718,7 +4712,7 @@
       <c r="G74" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H74" s="26" t="s">
+      <c r="H74" s="25" t="s">
         <v>129</v>
       </c>
       <c r="I74" s="6"/>
@@ -4739,7 +4733,7 @@
       <c r="X74" s="1"/>
       <c r="Y74" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="19.5">
       <c r="A75" s="5"/>
       <c r="B75" s="6" t="s">
         <v>11</v>
@@ -4750,7 +4744,7 @@
       <c r="D75" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E75" s="22" t="s">
+      <c r="E75" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F75" s="17" t="s">
@@ -4759,7 +4753,7 @@
       <c r="G75" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H75" s="26" t="s">
+      <c r="H75" s="25" t="s">
         <v>131</v>
       </c>
       <c r="I75" s="6"/>
@@ -4780,7 +4774,7 @@
       <c r="X75" s="1"/>
       <c r="Y75" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="19.5">
       <c r="A76" s="5"/>
       <c r="B76" s="6" t="s">
         <v>11</v>
@@ -4791,7 +4785,7 @@
       <c r="D76" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="E76" s="22" t="s">
+      <c r="E76" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F76" s="17" t="s">
@@ -4800,7 +4794,7 @@
       <c r="G76" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H76" s="27" t="s">
+      <c r="H76" s="26" t="s">
         <v>133</v>
       </c>
       <c r="I76" s="6"/>
@@ -4821,7 +4815,7 @@
       <c r="X76" s="1"/>
       <c r="Y76" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="19.5">
       <c r="A77" s="5"/>
       <c r="B77" s="6" t="s">
         <v>11</v>
@@ -4832,7 +4826,7 @@
       <c r="D77" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="E77" s="22" t="s">
+      <c r="E77" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F77" s="17" t="s">
@@ -4841,7 +4835,7 @@
       <c r="G77" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H77" s="26" t="s">
+      <c r="H77" s="25" t="s">
         <v>135</v>
       </c>
       <c r="I77" s="6"/>
@@ -4862,7 +4856,7 @@
       <c r="X77" s="1"/>
       <c r="Y77" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="19.5">
       <c r="A78" s="5"/>
       <c r="B78" s="6" t="s">
         <v>11</v>
@@ -4873,14 +4867,14 @@
       <c r="D78" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E78" s="22" t="s">
+      <c r="E78" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F78" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G78" s="6"/>
-      <c r="H78" s="27" t="s">
+      <c r="H78" s="26" t="s">
         <v>137</v>
       </c>
       <c r="I78" s="6"/>
@@ -4901,7 +4895,7 @@
       <c r="X78" s="1"/>
       <c r="Y78" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="19.5">
       <c r="A79" s="5"/>
       <c r="B79" s="6" t="s">
         <v>11</v>
@@ -4912,14 +4906,14 @@
       <c r="D79" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="E79" s="22" t="s">
+      <c r="E79" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F79" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G79" s="6"/>
-      <c r="H79" s="26" t="s">
+      <c r="H79" s="25" t="s">
         <v>139</v>
       </c>
       <c r="I79" s="6"/>
@@ -4940,7 +4934,7 @@
       <c r="X79" s="1"/>
       <c r="Y79" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="19.5">
       <c r="A80" s="5"/>
       <c r="B80" s="6" t="s">
         <v>11</v>
@@ -4951,7 +4945,7 @@
       <c r="D80" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="E80" s="22" t="s">
+      <c r="E80" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F80" s="17" t="s">
@@ -4960,7 +4954,7 @@
       <c r="G80" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H80" s="27" t="s">
+      <c r="H80" s="26" t="s">
         <v>141</v>
       </c>
       <c r="I80" s="6"/>
@@ -4981,7 +4975,7 @@
       <c r="X80" s="1"/>
       <c r="Y80" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="19.5">
       <c r="A81" s="5"/>
       <c r="B81" s="6" t="s">
         <v>11</v>
@@ -4992,14 +4986,14 @@
       <c r="D81" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="E81" s="22" t="s">
+      <c r="E81" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F81" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G81" s="6"/>
-      <c r="H81" s="27" t="s">
+      <c r="H81" s="26" t="s">
         <v>143</v>
       </c>
       <c r="I81" s="6"/>
@@ -5020,7 +5014,7 @@
       <c r="X81" s="1"/>
       <c r="Y81" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="19.5">
       <c r="A82" s="5"/>
       <c r="B82" s="6" t="s">
         <v>11</v>
@@ -5031,7 +5025,7 @@
       <c r="D82" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="E82" s="22" t="s">
+      <c r="E82" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F82" s="19" t="s">
@@ -5040,7 +5034,7 @@
       <c r="G82" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H82" s="27" t="s">
+      <c r="H82" s="26" t="s">
         <v>145</v>
       </c>
       <c r="I82" s="6"/>
@@ -5061,7 +5055,7 @@
       <c r="X82" s="1"/>
       <c r="Y82" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="19.5">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="2"/>
@@ -5088,7 +5082,7 @@
       <c r="X83" s="1"/>
       <c r="Y83" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="19.5">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="2"/>
@@ -5115,8 +5109,8 @@
       <c r="X84" s="1"/>
       <c r="Y84" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="17.25">
-      <c r="A85" s="28" t="s">
+    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="19.5">
+      <c r="A85" s="27" t="s">
         <v>146</v>
       </c>
       <c r="B85" s="6" t="s">
@@ -5128,7 +5122,7 @@
       <c r="D85" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="E85" s="22" t="s">
+      <c r="E85" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F85" s="15" t="s">
@@ -5137,7 +5131,7 @@
       <c r="G85" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H85" s="26" t="s">
+      <c r="H85" s="25" t="s">
         <v>148</v>
       </c>
       <c r="I85" s="6"/>
@@ -5158,7 +5152,7 @@
       <c r="X85" s="1"/>
       <c r="Y85" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="19.5">
       <c r="A86" s="5"/>
       <c r="B86" s="6" t="s">
         <v>11</v>
@@ -5169,7 +5163,7 @@
       <c r="D86" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="E86" s="22" t="s">
+      <c r="E86" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F86" s="15" t="s">
@@ -5178,7 +5172,7 @@
       <c r="G86" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H86" s="27" t="s">
+      <c r="H86" s="26" t="s">
         <v>150</v>
       </c>
       <c r="I86" s="6"/>
@@ -5199,7 +5193,7 @@
       <c r="X86" s="1"/>
       <c r="Y86" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="19.5">
       <c r="A87" s="5"/>
       <c r="B87" s="6" t="s">
         <v>11</v>
@@ -5210,7 +5204,7 @@
       <c r="D87" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="E87" s="22" t="s">
+      <c r="E87" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F87" s="15" t="s">
@@ -5219,7 +5213,7 @@
       <c r="G87" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H87" s="26" t="s">
+      <c r="H87" s="25" t="s">
         <v>152</v>
       </c>
       <c r="I87" s="6"/>
@@ -5240,7 +5234,7 @@
       <c r="X87" s="1"/>
       <c r="Y87" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="19.5">
       <c r="A88" s="5"/>
       <c r="B88" s="6" t="s">
         <v>11</v>
@@ -5251,7 +5245,7 @@
       <c r="D88" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="E88" s="22" t="s">
+      <c r="E88" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F88" s="15" t="s">
@@ -5260,7 +5254,7 @@
       <c r="G88" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H88" s="26" t="s">
+      <c r="H88" s="25" t="s">
         <v>154</v>
       </c>
       <c r="I88" s="6"/>
@@ -5281,7 +5275,7 @@
       <c r="X88" s="1"/>
       <c r="Y88" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="19.5">
       <c r="A89" s="5"/>
       <c r="B89" s="6" t="s">
         <v>11</v>
@@ -5292,7 +5286,7 @@
       <c r="D89" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="E89" s="22" t="s">
+      <c r="E89" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F89" s="15" t="s">
@@ -5301,7 +5295,7 @@
       <c r="G89" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H89" s="26" t="s">
+      <c r="H89" s="25" t="s">
         <v>156</v>
       </c>
       <c r="I89" s="6"/>
@@ -5322,7 +5316,7 @@
       <c r="X89" s="1"/>
       <c r="Y89" s="1"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="19.5">
       <c r="A90" s="5"/>
       <c r="B90" s="6" t="s">
         <v>11</v>
@@ -5333,14 +5327,14 @@
       <c r="D90" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="E90" s="22" t="s">
+      <c r="E90" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F90" s="15" t="s">
         <v>14</v>
       </c>
       <c r="G90" s="6"/>
-      <c r="H90" s="26" t="s">
+      <c r="H90" s="25" t="s">
         <v>158</v>
       </c>
       <c r="I90" s="6"/>
@@ -5372,14 +5366,14 @@
       <c r="D91" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="E91" s="22" t="s">
+      <c r="E91" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F91" s="15" t="s">
         <v>14</v>
       </c>
       <c r="G91" s="6"/>
-      <c r="H91" s="27" t="s">
+      <c r="H91" s="26" t="s">
         <v>160</v>
       </c>
       <c r="I91" s="6"/>
@@ -5420,7 +5414,7 @@
       <c r="G92" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H92" s="26" t="s">
+      <c r="H92" s="25" t="s">
         <v>162</v>
       </c>
       <c r="I92" s="6"/>
@@ -5452,7 +5446,7 @@
       <c r="D93" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="E93" s="22" t="s">
+      <c r="E93" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F93" s="17" t="s">
@@ -5461,7 +5455,7 @@
       <c r="G93" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H93" s="26" t="s">
+      <c r="H93" s="25" t="s">
         <v>164</v>
       </c>
       <c r="I93" s="6"/>
@@ -5493,7 +5487,7 @@
       <c r="D94" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="E94" s="22" t="s">
+      <c r="E94" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F94" s="17" t="s">
@@ -5502,7 +5496,7 @@
       <c r="G94" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H94" s="26" t="s">
+      <c r="H94" s="25" t="s">
         <v>166</v>
       </c>
       <c r="I94" s="6"/>
@@ -5534,7 +5528,7 @@
       <c r="D95" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="E95" s="22" t="s">
+      <c r="E95" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F95" s="17" t="s">
@@ -5543,7 +5537,7 @@
       <c r="G95" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H95" s="27" t="s">
+      <c r="H95" s="26" t="s">
         <v>168</v>
       </c>
       <c r="I95" s="6"/>
@@ -5575,7 +5569,7 @@
       <c r="D96" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="E96" s="22" t="s">
+      <c r="E96" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F96" s="17" t="s">
@@ -5584,7 +5578,7 @@
       <c r="G96" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H96" s="26" t="s">
+      <c r="H96" s="25" t="s">
         <v>170</v>
       </c>
       <c r="I96" s="6"/>
@@ -5616,14 +5610,14 @@
       <c r="D97" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E97" s="22" t="s">
+      <c r="E97" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F97" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G97" s="6"/>
-      <c r="H97" s="26" t="s">
+      <c r="H97" s="25" t="s">
         <v>172</v>
       </c>
       <c r="I97" s="6"/>
@@ -5655,7 +5649,7 @@
       <c r="D98" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="E98" s="22" t="s">
+      <c r="E98" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F98" s="17" t="s">
@@ -5664,7 +5658,7 @@
       <c r="G98" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H98" s="26" t="s">
+      <c r="H98" s="25" t="s">
         <v>174</v>
       </c>
       <c r="I98" s="6"/>
@@ -5696,7 +5690,7 @@
       <c r="D99" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="E99" s="22" t="s">
+      <c r="E99" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F99" s="19" t="s">
@@ -5705,7 +5699,7 @@
       <c r="G99" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H99" s="27" t="s">
+      <c r="H99" s="26" t="s">
         <v>176</v>
       </c>
       <c r="I99" s="6"/>
@@ -5781,7 +5775,7 @@
       <c r="Y101" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="17.25">
-      <c r="A102" s="28" t="s">
+      <c r="A102" s="27" t="s">
         <v>177</v>
       </c>
       <c r="B102" s="6" t="s">
@@ -5793,16 +5787,16 @@
       <c r="D102" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E102" s="22" t="s">
+      <c r="E102" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F102" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="G102" s="23" t="s">
+      <c r="G102" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="H102" s="27" t="s">
+      <c r="H102" s="26" t="s">
         <v>179</v>
       </c>
       <c r="I102" s="6"/>
@@ -5834,7 +5828,7 @@
       <c r="D103" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="E103" s="22" t="s">
+      <c r="E103" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F103" s="15" t="s">
@@ -5843,7 +5837,7 @@
       <c r="G103" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H103" s="27" t="s">
+      <c r="H103" s="26" t="s">
         <v>181</v>
       </c>
       <c r="I103" s="6"/>
@@ -5875,7 +5869,7 @@
       <c r="D104" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="E104" s="22" t="s">
+      <c r="E104" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F104" s="15" t="s">
@@ -5884,7 +5878,7 @@
       <c r="G104" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H104" s="27" t="s">
+      <c r="H104" s="26" t="s">
         <v>183</v>
       </c>
       <c r="I104" s="6"/>
@@ -5916,14 +5910,14 @@
       <c r="D105" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="E105" s="22" t="s">
+      <c r="E105" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F105" s="15" t="s">
         <v>14</v>
       </c>
       <c r="G105" s="6"/>
-      <c r="H105" s="26" t="s">
+      <c r="H105" s="25" t="s">
         <v>185</v>
       </c>
       <c r="I105" s="6"/>
@@ -5955,7 +5949,7 @@
       <c r="D106" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="E106" s="22" t="s">
+      <c r="E106" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F106" s="15" t="s">
@@ -5964,7 +5958,7 @@
       <c r="G106" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="H106" s="27" t="s">
+      <c r="H106" s="26" t="s">
         <v>188</v>
       </c>
       <c r="I106" s="6"/>
@@ -5996,7 +5990,7 @@
       <c r="D107" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="E107" s="22" t="s">
+      <c r="E107" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F107" s="15" t="s">
@@ -6005,7 +5999,7 @@
       <c r="G107" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H107" s="26" t="s">
+      <c r="H107" s="25" t="s">
         <v>190</v>
       </c>
       <c r="I107" s="6"/>
@@ -6037,7 +6031,7 @@
       <c r="D108" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="E108" s="22" t="s">
+      <c r="E108" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F108" s="15" t="s">
@@ -6046,7 +6040,7 @@
       <c r="G108" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H108" s="27" t="s">
+      <c r="H108" s="26" t="s">
         <v>192</v>
       </c>
       <c r="I108" s="6"/>
@@ -6078,7 +6072,7 @@
       <c r="D109" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="E109" s="22" t="s">
+      <c r="E109" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F109" s="15" t="s">
@@ -6087,7 +6081,7 @@
       <c r="G109" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H109" s="27" t="s">
+      <c r="H109" s="26" t="s">
         <v>194</v>
       </c>
       <c r="I109" s="6"/>
@@ -6119,14 +6113,14 @@
       <c r="D110" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="E110" s="22" t="s">
+      <c r="E110" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F110" s="15" t="s">
         <v>14</v>
       </c>
       <c r="G110" s="6"/>
-      <c r="H110" s="26" t="s">
+      <c r="H110" s="25" t="s">
         <v>196</v>
       </c>
       <c r="I110" s="6"/>
@@ -6158,7 +6152,7 @@
       <c r="D111" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="E111" s="22" t="s">
+      <c r="E111" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F111" s="15" t="s">
@@ -6167,7 +6161,7 @@
       <c r="G111" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H111" s="26" t="s">
+      <c r="H111" s="25" t="s">
         <v>198</v>
       </c>
       <c r="I111" s="6"/>
@@ -6199,14 +6193,14 @@
       <c r="D112" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="E112" s="22" t="s">
+      <c r="E112" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F112" s="15" t="s">
         <v>14</v>
       </c>
       <c r="G112" s="6"/>
-      <c r="H112" s="26" t="s">
+      <c r="H112" s="25" t="s">
         <v>200</v>
       </c>
       <c r="I112" s="6"/>
@@ -6238,7 +6232,7 @@
       <c r="D113" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="E113" s="22" t="s">
+      <c r="E113" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F113" s="17" t="s">
@@ -6247,7 +6241,7 @@
       <c r="G113" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H113" s="26" t="s">
+      <c r="H113" s="25" t="s">
         <v>202</v>
       </c>
       <c r="I113" s="6"/>
@@ -6279,14 +6273,14 @@
       <c r="D114" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="E114" s="22" t="s">
+      <c r="E114" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F114" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G114" s="6"/>
-      <c r="H114" s="26" t="s">
+      <c r="H114" s="25" t="s">
         <v>204</v>
       </c>
       <c r="I114" s="6"/>
@@ -6318,14 +6312,14 @@
       <c r="D115" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="E115" s="22" t="s">
+      <c r="E115" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F115" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G115" s="6"/>
-      <c r="H115" s="26" t="s">
+      <c r="H115" s="25" t="s">
         <v>206</v>
       </c>
       <c r="I115" s="6"/>
@@ -6357,7 +6351,7 @@
       <c r="D116" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="E116" s="22" t="s">
+      <c r="E116" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F116" s="17" t="s">
@@ -6366,7 +6360,7 @@
       <c r="G116" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H116" s="26" t="s">
+      <c r="H116" s="25" t="s">
         <v>208</v>
       </c>
       <c r="I116" s="6"/>
@@ -6398,7 +6392,7 @@
       <c r="D117" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="E117" s="22" t="s">
+      <c r="E117" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F117" s="17" t="s">
@@ -6407,7 +6401,7 @@
       <c r="G117" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H117" s="26" t="s">
+      <c r="H117" s="25" t="s">
         <v>210</v>
       </c>
       <c r="I117" s="6"/>
@@ -6439,7 +6433,7 @@
       <c r="D118" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="E118" s="22" t="s">
+      <c r="E118" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F118" s="17" t="s">
@@ -6448,7 +6442,7 @@
       <c r="G118" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H118" s="26" t="s">
+      <c r="H118" s="25" t="s">
         <v>212</v>
       </c>
       <c r="I118" s="6"/>
@@ -6480,7 +6474,7 @@
       <c r="D119" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="E119" s="22" t="s">
+      <c r="E119" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F119" s="17" t="s">
@@ -6489,7 +6483,7 @@
       <c r="G119" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H119" s="26" t="s">
+      <c r="H119" s="25" t="s">
         <v>214</v>
       </c>
       <c r="I119" s="6"/>
@@ -6521,14 +6515,14 @@
       <c r="D120" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="E120" s="22" t="s">
+      <c r="E120" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F120" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G120" s="6"/>
-      <c r="H120" s="27" t="s">
+      <c r="H120" s="26" t="s">
         <v>216</v>
       </c>
       <c r="I120" s="6"/>
@@ -6560,7 +6554,7 @@
       <c r="D121" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="E121" s="22" t="s">
+      <c r="E121" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F121" s="17" t="s">
@@ -6569,7 +6563,7 @@
       <c r="G121" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H121" s="27" t="s">
+      <c r="H121" s="26" t="s">
         <v>218</v>
       </c>
       <c r="I121" s="6"/>
@@ -6601,7 +6595,7 @@
       <c r="D122" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="E122" s="22" t="s">
+      <c r="E122" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F122" s="17" t="s">
@@ -6610,7 +6604,7 @@
       <c r="G122" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H122" s="27" t="s">
+      <c r="H122" s="26" t="s">
         <v>220</v>
       </c>
       <c r="I122" s="6"/>
@@ -6642,14 +6636,14 @@
       <c r="D123" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="E123" s="22" t="s">
+      <c r="E123" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F123" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G123" s="6"/>
-      <c r="H123" s="26" t="s">
+      <c r="H123" s="25" t="s">
         <v>222</v>
       </c>
       <c r="I123" s="6"/>
@@ -6681,14 +6675,14 @@
       <c r="D124" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="E124" s="22" t="s">
+      <c r="E124" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F124" s="19" t="s">
         <v>63</v>
       </c>
       <c r="G124" s="6"/>
-      <c r="H124" s="26" t="s">
+      <c r="H124" s="25" t="s">
         <v>224</v>
       </c>
       <c r="I124" s="6"/>
@@ -6720,14 +6714,14 @@
       <c r="D125" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="E125" s="22" t="s">
+      <c r="E125" s="21" t="s">
         <v>13</v>
       </c>
       <c r="F125" s="19" t="s">
         <v>63</v>
       </c>
       <c r="G125" s="6"/>
-      <c r="H125" s="26" t="s">
+      <c r="H125" s="25" t="s">
         <v>226</v>
       </c>
       <c r="I125" s="6"/>
@@ -6803,7 +6797,7 @@
       <c r="Y127" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="17.25">
-      <c r="A128" s="28" t="s">
+      <c r="A128" s="27" t="s">
         <v>227</v>
       </c>
       <c r="B128" s="6" t="s">
@@ -6822,7 +6816,7 @@
         <v>14</v>
       </c>
       <c r="G128" s="6"/>
-      <c r="H128" s="26" t="s">
+      <c r="H128" s="25" t="s">
         <v>229</v>
       </c>
       <c r="I128" s="6"/>
@@ -6863,7 +6857,7 @@
       <c r="G129" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H129" s="27" t="s">
+      <c r="H129" s="26" t="s">
         <v>231</v>
       </c>
       <c r="I129" s="6"/>
@@ -6904,7 +6898,7 @@
       <c r="G130" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H130" s="26" t="s">
+      <c r="H130" s="25" t="s">
         <v>233</v>
       </c>
       <c r="I130" s="6"/>
@@ -6945,7 +6939,7 @@
       <c r="G131" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H131" s="26" t="s">
+      <c r="H131" s="25" t="s">
         <v>235</v>
       </c>
       <c r="I131" s="6"/>
@@ -6986,7 +6980,7 @@
       <c r="G132" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H132" s="26" t="s">
+      <c r="H132" s="25" t="s">
         <v>237</v>
       </c>
       <c r="I132" s="6"/>
@@ -7027,7 +7021,7 @@
       <c r="G133" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H133" s="27" t="s">
+      <c r="H133" s="26" t="s">
         <v>239</v>
       </c>
       <c r="I133" s="6"/>
@@ -7068,7 +7062,7 @@
       <c r="G134" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H134" s="27" t="s">
+      <c r="H134" s="26" t="s">
         <v>241</v>
       </c>
       <c r="I134" s="6"/>
@@ -7109,7 +7103,7 @@
       <c r="G135" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H135" s="26" t="s">
+      <c r="H135" s="25" t="s">
         <v>243</v>
       </c>
       <c r="I135" s="6"/>
@@ -7150,7 +7144,7 @@
       <c r="G136" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H136" s="27" t="s">
+      <c r="H136" s="26" t="s">
         <v>245</v>
       </c>
       <c r="I136" s="6"/>
@@ -7189,7 +7183,7 @@
         <v>27</v>
       </c>
       <c r="G137" s="6"/>
-      <c r="H137" s="26" t="s">
+      <c r="H137" s="25" t="s">
         <v>247</v>
       </c>
       <c r="I137" s="6"/>
@@ -7230,7 +7224,7 @@
       <c r="G138" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H138" s="26" t="s">
+      <c r="H138" s="25" t="s">
         <v>249</v>
       </c>
       <c r="I138" s="6"/>
@@ -7271,7 +7265,7 @@
       <c r="G139" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H139" s="26" t="s">
+      <c r="H139" s="25" t="s">
         <v>251</v>
       </c>
       <c r="I139" s="6"/>
@@ -7312,7 +7306,7 @@
       <c r="G140" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H140" s="27" t="s">
+      <c r="H140" s="26" t="s">
         <v>253</v>
       </c>
       <c r="I140" s="6"/>
@@ -7351,7 +7345,7 @@
         <v>63</v>
       </c>
       <c r="G141" s="6"/>
-      <c r="H141" s="27" t="s">
+      <c r="H141" s="26" t="s">
         <v>255</v>
       </c>
       <c r="I141" s="6"/>
@@ -7392,7 +7386,7 @@
       <c r="G142" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H142" s="26" t="s">
+      <c r="H142" s="25" t="s">
         <v>257</v>
       </c>
       <c r="I142" s="6"/>
@@ -7468,7 +7462,7 @@
       <c r="Y144" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="17.25">
-      <c r="A145" s="28" t="s">
+      <c r="A145" s="27" t="s">
         <v>258</v>
       </c>
       <c r="B145" s="6" t="s">
@@ -7480,14 +7474,14 @@
       <c r="D145" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="E145" s="29" t="s">
+      <c r="E145" s="28" t="s">
         <v>260</v>
       </c>
       <c r="F145" s="15" t="s">
         <v>14</v>
       </c>
       <c r="G145" s="6"/>
-      <c r="H145" s="26" t="s">
+      <c r="H145" s="25" t="s">
         <v>261</v>
       </c>
       <c r="I145" s="6"/>
@@ -7519,14 +7513,14 @@
       <c r="D146" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="E146" s="29" t="s">
+      <c r="E146" s="28" t="s">
         <v>263</v>
       </c>
       <c r="F146" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G146" s="6"/>
-      <c r="H146" s="26" t="s">
+      <c r="H146" s="25" t="s">
         <v>264</v>
       </c>
       <c r="I146" s="6"/>
@@ -7558,14 +7552,14 @@
       <c r="D147" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="E147" s="29" t="s">
+      <c r="E147" s="28" t="s">
         <v>266</v>
       </c>
       <c r="F147" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G147" s="6"/>
-      <c r="H147" s="26" t="s">
+      <c r="H147" s="25" t="s">
         <v>267</v>
       </c>
       <c r="I147" s="6"/>
@@ -7597,14 +7591,14 @@
       <c r="D148" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="E148" s="29" t="s">
+      <c r="E148" s="28" t="s">
         <v>269</v>
       </c>
       <c r="F148" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G148" s="6"/>
-      <c r="H148" s="26" t="s">
+      <c r="H148" s="25" t="s">
         <v>270</v>
       </c>
       <c r="I148" s="6"/>
@@ -7636,14 +7630,14 @@
       <c r="D149" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="E149" s="29" t="s">
+      <c r="E149" s="28" t="s">
         <v>272</v>
       </c>
       <c r="F149" s="19" t="s">
         <v>63</v>
       </c>
       <c r="G149" s="6"/>
-      <c r="H149" s="26" t="s">
+      <c r="H149" s="25" t="s">
         <v>273</v>
       </c>
       <c r="I149" s="6"/>
@@ -7675,14 +7669,14 @@
       <c r="D150" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="E150" s="29" t="s">
+      <c r="E150" s="28" t="s">
         <v>275</v>
       </c>
       <c r="F150" s="19" t="s">
         <v>63</v>
       </c>
       <c r="G150" s="6"/>
-      <c r="H150" s="27" t="s">
+      <c r="H150" s="26" t="s">
         <v>276</v>
       </c>
       <c r="I150" s="6"/>
@@ -7758,7 +7752,7 @@
       <c r="Y152" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="17.25">
-      <c r="A153" s="28" t="s">
+      <c r="A153" s="27" t="s">
         <v>277</v>
       </c>
       <c r="B153" s="6" t="s">
@@ -7770,14 +7764,14 @@
       <c r="D153" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E153" s="29" t="s">
+      <c r="E153" s="28" t="s">
         <v>278</v>
       </c>
       <c r="F153" s="15" t="s">
         <v>14</v>
       </c>
       <c r="G153" s="6"/>
-      <c r="H153" s="26" t="s">
+      <c r="H153" s="25" t="s">
         <v>279</v>
       </c>
       <c r="I153" s="6"/>
@@ -7809,14 +7803,14 @@
       <c r="D154" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="E154" s="29" t="s">
+      <c r="E154" s="28" t="s">
         <v>281</v>
       </c>
       <c r="F154" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G154" s="6"/>
-      <c r="H154" s="26" t="s">
+      <c r="H154" s="25" t="s">
         <v>282</v>
       </c>
       <c r="I154" s="6"/>
@@ -7848,14 +7842,14 @@
       <c r="D155" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="E155" s="29" t="s">
+      <c r="E155" s="28" t="s">
         <v>284</v>
       </c>
       <c r="F155" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G155" s="6"/>
-      <c r="H155" s="27" t="s">
+      <c r="H155" s="26" t="s">
         <v>285</v>
       </c>
       <c r="I155" s="6"/>
@@ -7887,14 +7881,14 @@
       <c r="D156" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="E156" s="29" t="s">
+      <c r="E156" s="28" t="s">
         <v>287</v>
       </c>
       <c r="F156" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G156" s="6"/>
-      <c r="H156" s="26" t="s">
+      <c r="H156" s="25" t="s">
         <v>288</v>
       </c>
       <c r="I156" s="6"/>
@@ -7926,14 +7920,14 @@
       <c r="D157" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="E157" s="29" t="s">
+      <c r="E157" s="28" t="s">
         <v>290</v>
       </c>
       <c r="F157" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G157" s="6"/>
-      <c r="H157" s="27" t="s">
+      <c r="H157" s="26" t="s">
         <v>285</v>
       </c>
       <c r="I157" s="6"/>
@@ -7955,7 +7949,7 @@
       <c r="Y157" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="17.25">
-      <c r="A158" s="30"/>
+      <c r="A158" s="29"/>
       <c r="B158" s="1"/>
       <c r="C158" s="2"/>
       <c r="D158" s="1"/>
@@ -8009,7 +8003,7 @@
       <c r="Y159" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="17.25">
-      <c r="A160" s="28" t="s">
+      <c r="A160" s="27" t="s">
         <v>291</v>
       </c>
       <c r="B160" s="6" t="s">
@@ -8021,14 +8015,14 @@
       <c r="D160" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="E160" s="29" t="s">
+      <c r="E160" s="28" t="s">
         <v>293</v>
       </c>
       <c r="F160" s="15" t="s">
         <v>14</v>
       </c>
       <c r="G160" s="6"/>
-      <c r="H160" s="26" t="s">
+      <c r="H160" s="25" t="s">
         <v>294</v>
       </c>
       <c r="I160" s="6"/>
@@ -8060,7 +8054,7 @@
       <c r="D161" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="E161" s="31" t="s">
+      <c r="E161" s="30" t="s">
         <v>296</v>
       </c>
       <c r="F161" s="17" t="s">
@@ -8069,7 +8063,7 @@
       <c r="G161" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H161" s="26" t="s">
+      <c r="H161" s="25" t="s">
         <v>297</v>
       </c>
       <c r="I161" s="6"/>
@@ -8101,7 +8095,7 @@
       <c r="D162" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="E162" s="31" t="s">
+      <c r="E162" s="30" t="s">
         <v>296</v>
       </c>
       <c r="F162" s="17" t="s">
@@ -8110,7 +8104,7 @@
       <c r="G162" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H162" s="26" t="s">
+      <c r="H162" s="25" t="s">
         <v>299</v>
       </c>
       <c r="I162" s="6"/>
@@ -8142,14 +8136,14 @@
       <c r="D163" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="E163" s="29" t="s">
+      <c r="E163" s="28" t="s">
         <v>301</v>
       </c>
       <c r="F163" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G163" s="6"/>
-      <c r="H163" s="26" t="s">
+      <c r="H163" s="25" t="s">
         <v>299</v>
       </c>
       <c r="I163" s="6"/>
@@ -8181,14 +8175,14 @@
       <c r="D164" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="E164" s="29" t="s">
+      <c r="E164" s="28" t="s">
         <v>301</v>
       </c>
       <c r="F164" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G164" s="6"/>
-      <c r="H164" s="26" t="s">
+      <c r="H164" s="25" t="s">
         <v>303</v>
       </c>
       <c r="I164" s="6"/>
@@ -8220,14 +8214,14 @@
       <c r="D165" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="E165" s="29" t="s">
+      <c r="E165" s="28" t="s">
         <v>305</v>
       </c>
       <c r="F165" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G165" s="6"/>
-      <c r="H165" s="26" t="s">
+      <c r="H165" s="25" t="s">
         <v>306</v>
       </c>
       <c r="I165" s="6"/>
@@ -8259,14 +8253,14 @@
       <c r="D166" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="E166" s="29" t="s">
+      <c r="E166" s="28" t="s">
         <v>305</v>
       </c>
       <c r="F166" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G166" s="6"/>
-      <c r="H166" s="26" t="s">
+      <c r="H166" s="25" t="s">
         <v>308</v>
       </c>
       <c r="I166" s="6"/>
@@ -8298,14 +8292,14 @@
       <c r="D167" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="E167" s="29" t="s">
+      <c r="E167" s="28" t="s">
         <v>310</v>
       </c>
       <c r="F167" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G167" s="6"/>
-      <c r="H167" s="26" t="s">
+      <c r="H167" s="25" t="s">
         <v>311</v>
       </c>
       <c r="I167" s="6"/>
@@ -8337,14 +8331,14 @@
       <c r="D168" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="E168" s="29" t="s">
+      <c r="E168" s="28" t="s">
         <v>313</v>
       </c>
       <c r="F168" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G168" s="6"/>
-      <c r="H168" s="26" t="s">
+      <c r="H168" s="25" t="s">
         <v>314</v>
       </c>
       <c r="I168" s="6"/>
@@ -8376,14 +8370,14 @@
       <c r="D169" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="E169" s="29" t="s">
+      <c r="E169" s="28" t="s">
         <v>316</v>
       </c>
       <c r="F169" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G169" s="6"/>
-      <c r="H169" s="27" t="s">
+      <c r="H169" s="26" t="s">
         <v>317</v>
       </c>
       <c r="I169" s="6"/>
@@ -8415,14 +8409,14 @@
       <c r="D170" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="E170" s="29" t="s">
+      <c r="E170" s="28" t="s">
         <v>319</v>
       </c>
       <c r="F170" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G170" s="6"/>
-      <c r="H170" s="26" t="s">
+      <c r="H170" s="25" t="s">
         <v>320</v>
       </c>
       <c r="I170" s="6"/>
@@ -8454,14 +8448,14 @@
       <c r="D171" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="E171" s="29" t="s">
+      <c r="E171" s="28" t="s">
         <v>322</v>
       </c>
       <c r="F171" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G171" s="6"/>
-      <c r="H171" s="26" t="s">
+      <c r="H171" s="25" t="s">
         <v>323</v>
       </c>
       <c r="I171" s="6"/>
@@ -8493,14 +8487,14 @@
       <c r="D172" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="E172" s="29" t="s">
+      <c r="E172" s="28" t="s">
         <v>325</v>
       </c>
       <c r="F172" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G172" s="6"/>
-      <c r="H172" s="26" t="s">
+      <c r="H172" s="25" t="s">
         <v>326</v>
       </c>
       <c r="I172" s="6"/>
@@ -8532,14 +8526,14 @@
       <c r="D173" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="E173" s="29" t="s">
+      <c r="E173" s="28" t="s">
         <v>328</v>
       </c>
       <c r="F173" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G173" s="6"/>
-      <c r="H173" s="26" t="s">
+      <c r="H173" s="25" t="s">
         <v>329</v>
       </c>
       <c r="I173" s="6"/>
@@ -8571,14 +8565,14 @@
       <c r="D174" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E174" s="29" t="s">
+      <c r="E174" s="28" t="s">
         <v>330</v>
       </c>
       <c r="F174" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G174" s="6"/>
-      <c r="H174" s="26" t="s">
+      <c r="H174" s="25" t="s">
         <v>331</v>
       </c>
       <c r="I174" s="6"/>
@@ -8610,14 +8604,14 @@
       <c r="D175" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="E175" s="29" t="s">
+      <c r="E175" s="28" t="s">
         <v>333</v>
       </c>
       <c r="F175" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G175" s="6"/>
-      <c r="H175" s="26" t="s">
+      <c r="H175" s="25" t="s">
         <v>334</v>
       </c>
       <c r="I175" s="6"/>
@@ -8649,14 +8643,14 @@
       <c r="D176" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="E176" s="29" t="s">
+      <c r="E176" s="28" t="s">
         <v>336</v>
       </c>
       <c r="F176" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G176" s="6"/>
-      <c r="H176" s="26" t="s">
+      <c r="H176" s="25" t="s">
         <v>337</v>
       </c>
       <c r="I176" s="6"/>
@@ -8688,14 +8682,14 @@
       <c r="D177" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="E177" s="29" t="s">
+      <c r="E177" s="28" t="s">
         <v>339</v>
       </c>
       <c r="F177" s="19" t="s">
         <v>63</v>
       </c>
       <c r="G177" s="6"/>
-      <c r="H177" s="27" t="s">
+      <c r="H177" s="26" t="s">
         <v>340</v>
       </c>
       <c r="I177" s="6"/>
@@ -8727,14 +8721,14 @@
       <c r="D178" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="E178" s="29" t="s">
+      <c r="E178" s="28" t="s">
         <v>342</v>
       </c>
       <c r="F178" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G178" s="6"/>
-      <c r="H178" s="26" t="s">
+      <c r="H178" s="25" t="s">
         <v>343</v>
       </c>
       <c r="I178" s="6"/>
@@ -8766,14 +8760,14 @@
       <c r="D179" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="E179" s="29" t="s">
+      <c r="E179" s="28" t="s">
         <v>296</v>
       </c>
       <c r="F179" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G179" s="6"/>
-      <c r="H179" s="26" t="s">
+      <c r="H179" s="25" t="s">
         <v>345</v>
       </c>
       <c r="I179" s="6"/>
@@ -8805,14 +8799,14 @@
       <c r="D180" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="E180" s="29" t="s">
+      <c r="E180" s="28" t="s">
         <v>347</v>
       </c>
       <c r="F180" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G180" s="6"/>
-      <c r="H180" s="26" t="s">
+      <c r="H180" s="25" t="s">
         <v>348</v>
       </c>
       <c r="I180" s="6"/>
@@ -8844,14 +8838,14 @@
       <c r="D181" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="E181" s="29" t="s">
+      <c r="E181" s="28" t="s">
         <v>350</v>
       </c>
       <c r="F181" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G181" s="6"/>
-      <c r="H181" s="26" t="s">
+      <c r="H181" s="25" t="s">
         <v>351</v>
       </c>
       <c r="I181" s="6"/>
@@ -8883,14 +8877,14 @@
       <c r="D182" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="E182" s="29" t="s">
+      <c r="E182" s="28" t="s">
         <v>353</v>
       </c>
       <c r="F182" s="17" t="s">
         <v>27</v>
       </c>
       <c r="G182" s="6"/>
-      <c r="H182" s="27" t="s">
+      <c r="H182" s="26" t="s">
         <v>354</v>
       </c>
       <c r="I182" s="6"/>
@@ -8922,14 +8916,14 @@
       <c r="D183" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="E183" s="29" t="s">
+      <c r="E183" s="28" t="s">
         <v>356</v>
       </c>
       <c r="F183" s="19" t="s">
         <v>63</v>
       </c>
       <c r="G183" s="6"/>
-      <c r="H183" s="27" t="s">
+      <c r="H183" s="26" t="s">
         <v>357</v>
       </c>
       <c r="I183" s="6"/>
@@ -8961,14 +8955,14 @@
       <c r="D184" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="E184" s="29" t="s">
+      <c r="E184" s="28" t="s">
         <v>359</v>
       </c>
       <c r="F184" s="19" t="s">
         <v>63</v>
       </c>
       <c r="G184" s="6"/>
-      <c r="H184" s="27" t="s">
+      <c r="H184" s="26" t="s">
         <v>360</v>
       </c>
       <c r="I184" s="6"/>
@@ -9000,14 +8994,14 @@
       <c r="D185" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="E185" s="29" t="s">
+      <c r="E185" s="28" t="s">
         <v>313</v>
       </c>
       <c r="F185" s="19" t="s">
         <v>63</v>
       </c>
       <c r="G185" s="6"/>
-      <c r="H185" s="26" t="s">
+      <c r="H185" s="25" t="s">
         <v>362</v>
       </c>
       <c r="I185" s="6"/>
@@ -9083,7 +9077,7 @@
       <c r="Y187" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="17.25">
-      <c r="A188" s="28" t="s">
+      <c r="A188" s="27" t="s">
         <v>363</v>
       </c>
       <c r="B188" s="6" t="s">
@@ -9102,7 +9096,7 @@
         <v>14</v>
       </c>
       <c r="G188" s="6"/>
-      <c r="H188" s="26" t="s">
+      <c r="H188" s="25" t="s">
         <v>365</v>
       </c>
       <c r="I188" s="6"/>
@@ -9141,7 +9135,7 @@
         <v>27</v>
       </c>
       <c r="G189" s="6"/>
-      <c r="H189" s="26" t="s">
+      <c r="H189" s="25" t="s">
         <v>367</v>
       </c>
       <c r="I189" s="6"/>
@@ -9180,7 +9174,7 @@
         <v>27</v>
       </c>
       <c r="G190" s="6"/>
-      <c r="H190" s="27" t="s">
+      <c r="H190" s="26" t="s">
         <v>369</v>
       </c>
       <c r="I190" s="6"/>
@@ -9219,7 +9213,7 @@
         <v>27</v>
       </c>
       <c r="G191" s="6"/>
-      <c r="H191" s="27" t="s">
+      <c r="H191" s="26" t="s">
         <v>371</v>
       </c>
       <c r="I191" s="6"/>
@@ -9258,7 +9252,7 @@
         <v>27</v>
       </c>
       <c r="G192" s="6"/>
-      <c r="H192" s="26" t="s">
+      <c r="H192" s="25" t="s">
         <v>373</v>
       </c>
       <c r="I192" s="6"/>
@@ -9297,7 +9291,7 @@
         <v>27</v>
       </c>
       <c r="G193" s="6"/>
-      <c r="H193" s="26" t="s">
+      <c r="H193" s="25" t="s">
         <v>375</v>
       </c>
       <c r="I193" s="6"/>
@@ -9336,7 +9330,7 @@
         <v>27</v>
       </c>
       <c r="G194" s="6"/>
-      <c r="H194" s="26" t="s">
+      <c r="H194" s="25" t="s">
         <v>377</v>
       </c>
       <c r="I194" s="6"/>
@@ -9375,7 +9369,7 @@
         <v>27</v>
       </c>
       <c r="G195" s="6"/>
-      <c r="H195" s="27" t="s">
+      <c r="H195" s="26" t="s">
         <v>379</v>
       </c>
       <c r="I195" s="6"/>
@@ -9414,7 +9408,7 @@
         <v>27</v>
       </c>
       <c r="G196" s="6"/>
-      <c r="H196" s="26" t="s">
+      <c r="H196" s="25" t="s">
         <v>381</v>
       </c>
       <c r="I196" s="6"/>
@@ -9453,7 +9447,7 @@
         <v>27</v>
       </c>
       <c r="G197" s="6"/>
-      <c r="H197" s="26" t="s">
+      <c r="H197" s="25" t="s">
         <v>383</v>
       </c>
       <c r="I197" s="6"/>
@@ -9492,7 +9486,7 @@
         <v>27</v>
       </c>
       <c r="G198" s="6"/>
-      <c r="H198" s="27" t="s">
+      <c r="H198" s="26" t="s">
         <v>385</v>
       </c>
       <c r="I198" s="6"/>
@@ -9531,7 +9525,7 @@
         <v>27</v>
       </c>
       <c r="G199" s="6"/>
-      <c r="H199" s="26" t="s">
+      <c r="H199" s="25" t="s">
         <v>387</v>
       </c>
       <c r="I199" s="6"/>
@@ -9570,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="G200" s="6"/>
-      <c r="H200" s="26" t="s">
+      <c r="H200" s="25" t="s">
         <v>389</v>
       </c>
       <c r="I200" s="6"/>
@@ -9609,7 +9603,7 @@
         <v>27</v>
       </c>
       <c r="G201" s="6"/>
-      <c r="H201" s="26" t="s">
+      <c r="H201" s="25" t="s">
         <v>391</v>
       </c>
       <c r="I201" s="6"/>
@@ -9648,7 +9642,7 @@
         <v>27</v>
       </c>
       <c r="G202" s="6"/>
-      <c r="H202" s="27" t="s">
+      <c r="H202" s="26" t="s">
         <v>393</v>
       </c>
       <c r="I202" s="6"/>
@@ -9687,7 +9681,7 @@
         <v>63</v>
       </c>
       <c r="G203" s="6"/>
-      <c r="H203" s="27" t="s">
+      <c r="H203" s="26" t="s">
         <v>395</v>
       </c>
       <c r="I203" s="6"/>
@@ -9726,7 +9720,7 @@
         <v>63</v>
       </c>
       <c r="G204" s="6"/>
-      <c r="H204" s="27" t="s">
+      <c r="H204" s="26" t="s">
         <v>397</v>
       </c>
       <c r="I204" s="6"/>
@@ -9765,7 +9759,7 @@
         <v>63</v>
       </c>
       <c r="G205" s="6"/>
-      <c r="H205" s="27" t="s">
+      <c r="H205" s="26" t="s">
         <v>399</v>
       </c>
       <c r="I205" s="6"/>
@@ -9804,7 +9798,7 @@
         <v>63</v>
       </c>
       <c r="G206" s="6"/>
-      <c r="H206" s="26" t="s">
+      <c r="H206" s="25" t="s">
         <v>401</v>
       </c>
       <c r="I206" s="6"/>
@@ -9843,7 +9837,7 @@
         <v>63</v>
       </c>
       <c r="G207" s="6"/>
-      <c r="H207" s="26" t="s">
+      <c r="H207" s="25" t="s">
         <v>403</v>
       </c>
       <c r="I207" s="6"/>
@@ -9882,7 +9876,7 @@
         <v>63</v>
       </c>
       <c r="G208" s="6"/>
-      <c r="H208" s="27" t="s">
+      <c r="H208" s="26" t="s">
         <v>405</v>
       </c>
       <c r="I208" s="6"/>
@@ -9958,7 +9952,7 @@
       <c r="Y210" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="211" customHeight="1" ht="17.25">
-      <c r="A211" s="28" t="s">
+      <c r="A211" s="27" t="s">
         <v>406</v>
       </c>
       <c r="B211" s="6" t="s">
@@ -9977,7 +9971,7 @@
         <v>14</v>
       </c>
       <c r="G211" s="6"/>
-      <c r="H211" s="27" t="s">
+      <c r="H211" s="26" t="s">
         <v>408</v>
       </c>
       <c r="I211" s="6"/>
@@ -10016,7 +10010,7 @@
         <v>27</v>
       </c>
       <c r="G212" s="6"/>
-      <c r="H212" s="26" t="s">
+      <c r="H212" s="25" t="s">
         <v>410</v>
       </c>
       <c r="I212" s="6"/>
@@ -10055,7 +10049,7 @@
         <v>27</v>
       </c>
       <c r="G213" s="6"/>
-      <c r="H213" s="26" t="s">
+      <c r="H213" s="25" t="s">
         <v>412</v>
       </c>
       <c r="I213" s="6"/>
@@ -10094,7 +10088,7 @@
         <v>27</v>
       </c>
       <c r="G214" s="6"/>
-      <c r="H214" s="26" t="s">
+      <c r="H214" s="25" t="s">
         <v>414</v>
       </c>
       <c r="I214" s="6"/>
@@ -10133,7 +10127,7 @@
         <v>27</v>
       </c>
       <c r="G215" s="6"/>
-      <c r="H215" s="26" t="s">
+      <c r="H215" s="25" t="s">
         <v>416</v>
       </c>
       <c r="I215" s="6"/>
@@ -10172,7 +10166,7 @@
         <v>63</v>
       </c>
       <c r="G216" s="6"/>
-      <c r="H216" s="26" t="s">
+      <c r="H216" s="25" t="s">
         <v>418</v>
       </c>
       <c r="I216" s="6"/>

</xml_diff>